<commit_message>
fix: sample create wallet container loads file (#12582)
</commit_message>
<xml_diff>
--- a/public/files/sample_create_wallet_container_loads.xlsx
+++ b/public/files/sample_create_wallet_container_loads.xlsx
@@ -22,7 +22,7 @@
     <t>Amount (In Paise)</t>
   </si>
   <si>
-    <t>Reference ID(Optional)</t>
+    <t>Reference ID (Optional)</t>
   </si>
   <si>
     <t>Description (Optional)</t>
@@ -38,7 +38,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -48,11 +48,6 @@
       <sz val="12"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Arial"/>
     </font>
     <font>
       <sz val="15"/>
@@ -163,25 +158,25 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -220,10 +215,10 @@
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="5E5E5E"/>
+        <a:srgbClr val="A7A7A7"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="D5D5D5"/>
+        <a:srgbClr val="535353"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="00A2FF"/>
@@ -400,11 +395,14 @@
     <a:spDef>
       <a:spPr>
         <a:solidFill>
-          <a:srgbClr val="000000"/>
+          <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -413,33 +411,33 @@
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="ctr" defTabSz="584200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
-          <a:lnSpc>
-            <a:spcPct val="100000"/>
-          </a:lnSpc>
-          <a:spcBef>
-            <a:spcPts val="0"/>
-          </a:spcBef>
-          <a:spcAft>
-            <a:spcPts val="0"/>
-          </a:spcAft>
-          <a:buClrTx/>
-          <a:buSzTx/>
-          <a:buFontTx/>
-          <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1200" u="none" kumimoji="0" normalizeH="0">
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:uFillTx/>
-            <a:latin typeface="Helvetica Neue Medium"/>
-            <a:ea typeface="Helvetica Neue Medium"/>
-            <a:cs typeface="Helvetica Neue Medium"/>
-            <a:sym typeface="Helvetica Neue Medium"/>
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -678,12 +676,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
-            <a:srgbClr val="000000"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="400000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -964,7 +962,7 @@
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="457200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
           <a:lnSpc>
             <a:spcPct val="100000"/>
           </a:lnSpc>
@@ -1238,7 +1236,7 @@
     <col min="1" max="1" width="17.3516" style="1" customWidth="1"/>
     <col min="2" max="2" width="21.3516" style="1" customWidth="1"/>
     <col min="3" max="3" width="16.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.4141" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.5" style="1" customWidth="1"/>
     <col min="5" max="6" width="19.5" style="1" customWidth="1"/>
     <col min="7" max="16384" width="12.6719" style="1" customWidth="1"/>
   </cols>

</xml_diff>